<commit_message>
Calidad: revisar las coincidencias débiles y probar con el ejemplo cada cambio del método
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ejemplo/resultado-esperado.xlsx
+++ b/ejemplo/resultado-esperado.xlsx
@@ -806,36 +806,36 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>0001-00000001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Lucía Fernández</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Referencia</t>
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>0001-00000006</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Julián Castro</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Aproximado (fecha + importe)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0001-00000002</t>
+          <t>0001-00000004</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Martín Gómez</t>
+          <t>Pablo Rodríguez</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Referencia con un dígito de menos</t>
+          <t>Nombre + importe</t>
         </is>
       </c>
     </row>
@@ -859,51 +859,51 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0001-00000004</t>
+          <t>0001-00000005</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pablo Rodríguez</t>
+          <t>Carla Díaz</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nombre + importe</t>
+          <t>Consumidor final por referencia</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0001-00000005</t>
+          <t>0001-00000002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Carla Díaz</t>
+          <t>Martín Gómez</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Consumidor final por referencia</t>
+          <t>Referencia con un dígito de menos</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>0001-00000006</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Julián Castro</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Aproximado (fecha + importe)</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0001-00000001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Lucía Fernández</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Referencia</t>
         </is>
       </c>
     </row>

</xml_diff>